<commit_message>
Atualiza relatorios de quimicos
</commit_message>
<xml_diff>
--- a/data-source/COMPRASQUIMICOS.xlsx
+++ b/data-source/COMPRASQUIMICOS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/QUIMICOS-ANALISE/data-source/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\impre\Downloads\QUIMICOS-ANALISE-QUIMICOS-V3\data-source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A87165D6-8DD7-4C3E-B395-713FA98E4A3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A64F101C-86C4-47A2-AE7F-5B799B46F906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,25 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Planilha!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="15">
   <si>
     <t>Núm.OC</t>
   </si>
@@ -62,6 +75,12 @@
   </si>
   <si>
     <t>PIGMENTO HP-H300S YELLOW CHINA</t>
+  </si>
+  <si>
+    <t>SOLVENTE DMF (NACIONAL)</t>
+  </si>
+  <si>
+    <t>SOLVENTE</t>
   </si>
 </sst>
 </file>
@@ -70,8 +89,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[Blue]###########0;[Red]\-###########0"/>
-    <numFmt numFmtId="166" formatCode="[Blue]###,###,###,##0.000;[Red]\-###,###,###,##0.000"/>
-    <numFmt numFmtId="167" formatCode="[Blue]###,###,###,##0.0000;[Red]\-###,###,###,##0.0000"/>
+    <numFmt numFmtId="165" formatCode="[Blue]###,###,###,##0.000;[Red]\-###,###,###,##0.000"/>
+    <numFmt numFmtId="166" formatCode="[Blue]###,###,###,##0.0000;[Red]\-###,###,###,##0.0000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -133,8 +152,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -473,7 +492,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
@@ -642,6 +661,162 @@
         <v>46344</v>
       </c>
     </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>1042</v>
+      </c>
+      <c r="B7" s="3">
+        <v>8329</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="3">
+        <v>9</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="4">
+        <v>950</v>
+      </c>
+      <c r="G7" s="5">
+        <v>1.21</v>
+      </c>
+      <c r="H7" s="6">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>1042</v>
+      </c>
+      <c r="B8" s="3">
+        <v>8329</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="3">
+        <v>9</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="4">
+        <v>2850</v>
+      </c>
+      <c r="G8" s="5">
+        <v>1.21</v>
+      </c>
+      <c r="H8" s="6">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>1617</v>
+      </c>
+      <c r="B9" s="3">
+        <v>8329</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="3">
+        <v>9</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4">
+        <v>2850</v>
+      </c>
+      <c r="G9" s="5">
+        <v>1.75</v>
+      </c>
+      <c r="H9" s="6">
+        <v>46294</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>1617</v>
+      </c>
+      <c r="B10" s="3">
+        <v>8329</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="3">
+        <v>9</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="4">
+        <v>2850</v>
+      </c>
+      <c r="G10" s="5">
+        <v>1.75</v>
+      </c>
+      <c r="H10" s="6">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>1617</v>
+      </c>
+      <c r="B11" s="3">
+        <v>8329</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="3">
+        <v>9</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="4">
+        <v>2850</v>
+      </c>
+      <c r="G11" s="5">
+        <v>1.75</v>
+      </c>
+      <c r="H11" s="6">
+        <v>46356</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
+        <v>1617</v>
+      </c>
+      <c r="B12" s="3">
+        <v>8329</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="3">
+        <v>9</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="4">
+        <v>3800</v>
+      </c>
+      <c r="G12" s="5">
+        <v>1.75</v>
+      </c>
+      <c r="H12" s="6">
+        <v>46366</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>